<commit_message>
final report and register
</commit_message>
<xml_diff>
--- a/spreadsheet/Requirement_register_updated.xlsx
+++ b/spreadsheet/Requirement_register_updated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\NMBU\semester_2\inf203\Inf-203\spreadsheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{019A6F04-0370-4046-8BA4-F23F9825E9EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38F5BBAC-A605-4286-9A16-D1D585B0AFB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C6D9093C-116D-4EBF-B38E-58A8BAA2683C}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="67">
   <si>
     <t>Label</t>
   </si>
@@ -92,9 +92,6 @@
     <t>Must</t>
   </si>
   <si>
-    <t>Muust</t>
-  </si>
-  <si>
     <t>Izza</t>
   </si>
   <si>
@@ -122,9 +119,6 @@
     <t>Martin</t>
   </si>
   <si>
-    <t>Safely handle messy or incomplete JSON-LD without breaking the import process(MARTIN CHECK IF YOU DO THIS IN TASK 11)</t>
-  </si>
-  <si>
     <t>User Story 2.4</t>
   </si>
   <si>
@@ -242,10 +236,10 @@
     <t>Philip,Martin,Izza</t>
   </si>
   <si>
-    <t>Validated</t>
-  </si>
-  <si>
     <t>I want regression and acceptance tests that validate full end‑to‑end workflows so that I can detect breaking changes early and confirm that the system meets user‑level expectations.</t>
+  </si>
+  <si>
+    <t>Safely handle messy or incomplete JSON-LD without breaking the import process</t>
   </si>
 </sst>
 </file>
@@ -681,9 +675,7 @@
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
-        <v>67</v>
-      </c>
+      <c r="I1" s="3"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -707,7 +699,7 @@
         <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
@@ -716,13 +708,13 @@
         <v>16</v>
       </c>
       <c r="F3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -733,22 +725,22 @@
         <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -759,361 +751,361 @@
         <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D5" t="s">
         <v>8</v>
       </c>
       <c r="E5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" t="s">
         <v>17</v>
       </c>
-      <c r="F5" t="s">
-        <v>18</v>
-      </c>
       <c r="G5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B7" t="s">
         <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B8" t="s">
         <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E8" t="s">
         <v>16</v>
       </c>
       <c r="F8" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="G8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B9" t="s">
         <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E9" t="s">
         <v>16</v>
       </c>
       <c r="F9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" t="s">
         <v>23</v>
       </c>
-      <c r="B10" t="s">
-        <v>12</v>
-      </c>
-      <c r="C10" t="s">
-        <v>52</v>
-      </c>
-      <c r="D10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" t="s">
-        <v>24</v>
-      </c>
       <c r="F10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B11" t="s">
         <v>12</v>
       </c>
       <c r="C11" t="s">
-        <v>27</v>
+        <v>66</v>
       </c>
       <c r="D11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E11" t="s">
         <v>16</v>
       </c>
       <c r="F11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B12" t="s">
         <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F12" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="G12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B14" t="s">
         <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D14" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B15" t="s">
         <v>12</v>
       </c>
       <c r="C15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D15" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E15" t="s">
         <v>16</v>
       </c>
       <c r="F15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B16" t="s">
         <v>12</v>
       </c>
       <c r="C16" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D16" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E16" t="s">
         <v>16</v>
       </c>
       <c r="F16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G16" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B17" t="s">
         <v>12</v>
       </c>
       <c r="C17" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D17" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E17" t="s">
         <v>16</v>
       </c>
       <c r="F17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B18" t="s">
         <v>12</v>
       </c>
       <c r="C18" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D18" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E18" t="s">
         <v>16</v>
       </c>
       <c r="F18" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="G18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B19" t="s">
         <v>12</v>
       </c>
       <c r="C19" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D19" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E19" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F19" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="G19" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H19" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B21" t="s">
         <v>12</v>
       </c>
       <c r="C21" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D21" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B22" t="s">
         <v>12</v>
       </c>
       <c r="C22" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D22" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E22" t="s">
         <v>16</v>
       </c>
       <c r="F22" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G22" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B23" t="s">
         <v>15</v>
       </c>
       <c r="C23" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D23" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E23" t="s">
         <v>16</v>
@@ -1121,68 +1113,68 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B25" t="s">
         <v>12</v>
       </c>
       <c r="C25" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D25" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B26" t="s">
         <v>12</v>
       </c>
       <c r="C26" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D26" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E26" t="s">
         <v>16</v>
       </c>
       <c r="F26" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="G26" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H26" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B27" t="s">
         <v>12</v>
       </c>
       <c r="C27" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D27" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E27" t="s">
         <v>16</v>
       </c>
       <c r="F27" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="G27" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H27" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>